<commit_message>
Group B: 6801-L / 6801-LL folded into 6801 (extra length = ORB hex arm, measured on the Brennan STEPs): +11 configurations, old 39 unchanged
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Sbz7LkX6Jr9QuSxTU76dzT
</commit_message>
<xml_diff>
--- a/tools/_out/groupB_20261021/stage/04_DESIGN_TABLES/DesignTable_6801L.xlsx
+++ b/tools/_out/groupB_20261021/stage/04_DESIGN_TABLES/DesignTable_6801L.xlsx
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S22"/>
+  <dimension ref="A1:U22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -518,42 +518,52 @@
           <t>ORB_GRVW@DRIVE</t>
         </is>
       </c>
-      <c r="L2" s="2" t="inlineStr">
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>ORB_I3@DRIVE</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>ORB_THDL@DRIVE</t>
+        </is>
+      </c>
+      <c r="N2" s="2" t="inlineStr">
         <is>
           <t>$PRP@PartNo</t>
         </is>
       </c>
-      <c r="M2" s="2" t="inlineStr">
+      <c r="O2" s="2" t="inlineStr">
         <is>
           <t>$PRP@Threads</t>
         </is>
       </c>
-      <c r="N2" s="2" t="inlineStr">
+      <c r="P2" s="2" t="inlineStr">
         <is>
           <t>$PRP@DataStatus</t>
         </is>
       </c>
-      <c r="O2" s="2" t="inlineStr">
+      <c r="Q2" s="2" t="inlineStr">
         <is>
           <t>$PRP@AxialSource</t>
         </is>
       </c>
-      <c r="P2" s="2" t="inlineStr">
+      <c r="R2" s="2" t="inlineStr">
         <is>
           <t>$COMMENT</t>
         </is>
       </c>
-      <c r="Q2" t="inlineStr">
+      <c r="S2" t="inlineStr">
         <is>
           <t>$PRP@ScopeAction</t>
         </is>
       </c>
-      <c r="R2" t="inlineStr">
+      <c r="T2" t="inlineStr">
         <is>
           <t>$PRP@OMiSKU</t>
         </is>
       </c>
-      <c r="S2" t="inlineStr">
+      <c r="U2" t="inlineStr">
         <is>
           <t>$PRP@DimSource</t>
         </is>
@@ -595,33 +605,43 @@
       <c r="K3" s="3" t="n">
         <v>0.075</v>
       </c>
-      <c r="L3" s="3" t="inlineStr">
+      <c r="L3" t="n">
+        <v>0.73</v>
+      </c>
+      <c r="M3" t="n">
+        <v>0.265</v>
+      </c>
+      <c r="N3" s="3" t="inlineStr">
         <is>
           <t>6801-L-04-04-NWO-FG</t>
         </is>
       </c>
-      <c r="M3" s="3" t="inlineStr">
+      <c r="O3" s="3" t="inlineStr">
         <is>
           <t>7/16-20 (JIC) x 7/16-20 (male ORB) long pattern</t>
         </is>
       </c>
-      <c r="N3" s="3" t="inlineStr">
+      <c r="P3" s="3" t="inlineStr">
         <is>
           <t>ASSUMED</t>
         </is>
       </c>
-      <c r="O3" s="3" t="inlineStr">
-        <is>
-          <t>Air-Way s135 only (double-pass 18 rows); M matches verified 6801 family; JIC/ORB ends inherit library verification</t>
-        </is>
-      </c>
-      <c r="P3" s="3" t="inlineStr"/>
-      <c r="Q3" t="inlineStr">
+      <c r="Q3" s="3" t="inlineStr">
+        <is>
+          <t>Air-Way s135 only (double-pass 18 rows); M matches verified 6801 family; JIC/ORB ends inherit library verification | ORB_I3 0.73 = Air-Way 6801 rows of the -04 ORB size (A5; I3 = Brennan 6801 / 6801-L / 6801-LL STEPs at -08) | ORB_THDL 0.265 = Air-Way 6801 rows of the -04 ORB size (A5; I3 = Brennan 6801 / 6801-L / 6801-LL STEPs at -08)</t>
+        </is>
+      </c>
+      <c r="R3" s="3" t="inlineStr">
+        <is>
+          <t>Brennan CAD record ORB leg M7 1.54 vs Air-Way M11 1.19 - built to Air-Way (Air-Way first; tell the user / OMi)</t>
+        </is>
+      </c>
+      <c r="S3" t="inlineStr">
         <is>
           <t>BUILD</t>
         </is>
       </c>
-      <c r="R3" t="inlineStr">
+      <c r="T3" t="inlineStr">
         <is>
           <t>6801-L-04-04-NWO-FG</t>
         </is>
@@ -663,32 +683,32 @@
       <c r="K4" s="3" t="n">
         <v>0.083</v>
       </c>
-      <c r="L4" s="3" t="inlineStr">
+      <c r="N4" s="3" t="inlineStr">
         <is>
           <t>6801-L-04-06-NWO</t>
         </is>
       </c>
-      <c r="M4" s="3" t="inlineStr">
+      <c r="O4" s="3" t="inlineStr">
         <is>
           <t>7/16-20 (JIC) x 9/16-18 (male ORB) long pattern</t>
         </is>
       </c>
-      <c r="N4" s="3" t="inlineStr">
+      <c r="P4" s="3" t="inlineStr">
         <is>
           <t>ASSUMED</t>
         </is>
       </c>
-      <c r="O4" s="3" t="inlineStr">
+      <c r="Q4" s="3" t="inlineStr">
         <is>
           <t>Air-Way s135 only (double-pass 18 rows); M matches verified 6801 family; JIC/ORB ends inherit library verification</t>
         </is>
       </c>
-      <c r="P4" s="3" t="inlineStr">
+      <c r="R4" s="3" t="inlineStr">
         <is>
           <t>DROP: no matching OMi SKU in catalog feed (2026-09-23)</t>
         </is>
       </c>
-      <c r="Q4" t="inlineStr">
+      <c r="S4" t="inlineStr">
         <is>
           <t>DROP</t>
         </is>
@@ -730,33 +750,39 @@
       <c r="K5" s="3" t="n">
         <v>0.083</v>
       </c>
-      <c r="L5" s="3" t="inlineStr">
+      <c r="L5" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="M5" t="n">
+        <v>0.312</v>
+      </c>
+      <c r="N5" s="3" t="inlineStr">
         <is>
           <t>6801-L-06-06-NWO-FG</t>
         </is>
       </c>
-      <c r="M5" s="3" t="inlineStr">
+      <c r="O5" s="3" t="inlineStr">
         <is>
           <t>9/16-18 (JIC) x 9/16-18 (male ORB) long pattern</t>
         </is>
       </c>
-      <c r="N5" s="3" t="inlineStr">
+      <c r="P5" s="3" t="inlineStr">
         <is>
           <t>ASSUMED</t>
         </is>
       </c>
-      <c r="O5" s="3" t="inlineStr">
-        <is>
-          <t>Air-Way s135 only (double-pass 18 rows); M matches verified 6801 family; JIC/ORB ends inherit library verification</t>
-        </is>
-      </c>
-      <c r="P5" s="3" t="inlineStr"/>
-      <c r="Q5" t="inlineStr">
+      <c r="Q5" s="3" t="inlineStr">
+        <is>
+          <t>Air-Way s135 only (double-pass 18 rows); M matches verified 6801 family; JIC/ORB ends inherit library verification | ORB_I3 0.75 = Air-Way 6801 rows of the -06 ORB size (A5; I3 = Brennan 6801 / 6801-L / 6801-LL STEPs at -08) | ORB_THDL 0.312 = Air-Way 6801 rows of the -06 ORB size (A5; I3 = Brennan 6801 / 6801-L / 6801-LL STEPs at -08)</t>
+        </is>
+      </c>
+      <c r="R5" s="3" t="inlineStr"/>
+      <c r="S5" t="inlineStr">
         <is>
           <t>BUILD</t>
         </is>
       </c>
-      <c r="R5" t="inlineStr">
+      <c r="T5" t="inlineStr">
         <is>
           <t>6801-L-06-06-NWO-FG</t>
         </is>
@@ -798,32 +824,32 @@
       <c r="K6" s="3" t="n">
         <v>0.083</v>
       </c>
-      <c r="L6" s="3" t="inlineStr">
+      <c r="N6" s="3" t="inlineStr">
         <is>
           <t>6801-L-06-06-NWO</t>
         </is>
       </c>
-      <c r="M6" s="3" t="inlineStr">
+      <c r="O6" s="3" t="inlineStr">
         <is>
           <t>9/16-18 (JIC) x 9/16-18 (male ORB) long pattern</t>
         </is>
       </c>
-      <c r="N6" s="3" t="inlineStr">
+      <c r="P6" s="3" t="inlineStr">
         <is>
           <t>ASSUMED</t>
         </is>
       </c>
-      <c r="O6" s="3" t="inlineStr">
+      <c r="Q6" s="3" t="inlineStr">
         <is>
           <t>Air-Way s135 only (double-pass 18 rows); M matches verified 6801 family; JIC/ORB ends inherit library verification</t>
         </is>
       </c>
-      <c r="P6" s="3" t="inlineStr">
+      <c r="R6" s="3" t="inlineStr">
         <is>
           <t>DROP: no matching OMi SKU in catalog feed (2026-09-23)</t>
         </is>
       </c>
-      <c r="Q6" t="inlineStr">
+      <c r="S6" t="inlineStr">
         <is>
           <t>DROP</t>
         </is>
@@ -865,32 +891,32 @@
       <c r="K7" s="3" t="n">
         <v>0.094</v>
       </c>
-      <c r="L7" s="3" t="inlineStr">
+      <c r="N7" s="3" t="inlineStr">
         <is>
           <t>6801-L-06-08-NWO</t>
         </is>
       </c>
-      <c r="M7" s="3" t="inlineStr">
+      <c r="O7" s="3" t="inlineStr">
         <is>
           <t>9/16-18 (JIC) x 3/4-16 (male ORB) long pattern</t>
         </is>
       </c>
-      <c r="N7" s="3" t="inlineStr">
+      <c r="P7" s="3" t="inlineStr">
         <is>
           <t>ASSUMED</t>
         </is>
       </c>
-      <c r="O7" s="3" t="inlineStr">
+      <c r="Q7" s="3" t="inlineStr">
         <is>
           <t>Air-Way s135 only (double-pass 18 rows); M matches verified 6801 family; JIC/ORB ends inherit library verification</t>
         </is>
       </c>
-      <c r="P7" s="3" t="inlineStr">
+      <c r="R7" s="3" t="inlineStr">
         <is>
           <t>DROP: no matching OMi SKU in catalog feed (2026-09-23)</t>
         </is>
       </c>
-      <c r="Q7" t="inlineStr">
+      <c r="S7" t="inlineStr">
         <is>
           <t>DROP</t>
         </is>
@@ -932,32 +958,32 @@
       <c r="K8" s="3" t="n">
         <v>0.107</v>
       </c>
-      <c r="L8" s="3" t="inlineStr">
+      <c r="N8" s="3" t="inlineStr">
         <is>
           <t>6801-L-06-10-NWO</t>
         </is>
       </c>
-      <c r="M8" s="3" t="inlineStr">
+      <c r="O8" s="3" t="inlineStr">
         <is>
           <t>9/16-18 (JIC) x 7/8-14 (male ORB) long pattern</t>
         </is>
       </c>
-      <c r="N8" s="3" t="inlineStr">
+      <c r="P8" s="3" t="inlineStr">
         <is>
           <t>ASSUMED</t>
         </is>
       </c>
-      <c r="O8" s="3" t="inlineStr">
+      <c r="Q8" s="3" t="inlineStr">
         <is>
           <t>Air-Way s135 only (double-pass 18 rows); M matches verified 6801 family; JIC/ORB ends inherit library verification</t>
         </is>
       </c>
-      <c r="P8" s="3" t="inlineStr">
+      <c r="R8" s="3" t="inlineStr">
         <is>
           <t>DROP: no matching OMi SKU in catalog feed (2026-09-23)</t>
         </is>
       </c>
-      <c r="Q8" t="inlineStr">
+      <c r="S8" t="inlineStr">
         <is>
           <t>DROP</t>
         </is>
@@ -999,32 +1025,32 @@
       <c r="K9" s="3" t="n">
         <v>0.075</v>
       </c>
-      <c r="L9" s="3" t="inlineStr">
+      <c r="N9" s="3" t="inlineStr">
         <is>
           <t>6801-L-08-05-NWO-FG</t>
         </is>
       </c>
-      <c r="M9" s="3" t="inlineStr">
+      <c r="O9" s="3" t="inlineStr">
         <is>
           <t>3/4-16 (JIC) x 1/2-20 (male ORB) long pattern</t>
         </is>
       </c>
-      <c r="N9" s="3" t="inlineStr">
+      <c r="P9" s="3" t="inlineStr">
         <is>
           <t>ASSUMED</t>
         </is>
       </c>
-      <c r="O9" s="3" t="inlineStr">
+      <c r="Q9" s="3" t="inlineStr">
         <is>
           <t>Air-Way s135 only (double-pass 18 rows); M matches verified 6801 family; JIC/ORB ends inherit library verification</t>
         </is>
       </c>
-      <c r="P9" s="3" t="inlineStr">
+      <c r="R9" s="3" t="inlineStr">
         <is>
           <t>DROP: no matching OMi SKU in catalog feed (2026-09-23)</t>
         </is>
       </c>
-      <c r="Q9" t="inlineStr">
+      <c r="S9" t="inlineStr">
         <is>
           <t>DROP</t>
         </is>
@@ -1066,32 +1092,32 @@
       <c r="K10" s="3" t="n">
         <v>0.083</v>
       </c>
-      <c r="L10" s="3" t="inlineStr">
+      <c r="N10" s="3" t="inlineStr">
         <is>
           <t>6801-L-08-06-NWO</t>
         </is>
       </c>
-      <c r="M10" s="3" t="inlineStr">
+      <c r="O10" s="3" t="inlineStr">
         <is>
           <t>3/4-16 (JIC) x 9/16-18 (male ORB) long pattern</t>
         </is>
       </c>
-      <c r="N10" s="3" t="inlineStr">
+      <c r="P10" s="3" t="inlineStr">
         <is>
           <t>ASSUMED</t>
         </is>
       </c>
-      <c r="O10" s="3" t="inlineStr">
+      <c r="Q10" s="3" t="inlineStr">
         <is>
           <t>Air-Way s135 only (double-pass 18 rows); M matches verified 6801 family; JIC/ORB ends inherit library verification</t>
         </is>
       </c>
-      <c r="P10" s="3" t="inlineStr">
+      <c r="R10" s="3" t="inlineStr">
         <is>
           <t>DROP: no matching OMi SKU in catalog feed (2026-09-23)</t>
         </is>
       </c>
-      <c r="Q10" t="inlineStr">
+      <c r="S10" t="inlineStr">
         <is>
           <t>DROP</t>
         </is>
@@ -1133,33 +1159,43 @@
       <c r="K11" s="3" t="n">
         <v>0.094</v>
       </c>
-      <c r="L11" s="3" t="inlineStr">
+      <c r="L11" t="n">
+        <v>0.86</v>
+      </c>
+      <c r="M11" t="n">
+        <v>0.344</v>
+      </c>
+      <c r="N11" s="3" t="inlineStr">
         <is>
           <t>6801-L-08-08-NWO-FG</t>
         </is>
       </c>
-      <c r="M11" s="3" t="inlineStr">
+      <c r="O11" s="3" t="inlineStr">
         <is>
           <t>3/4-16 (JIC) x 3/4-16 (male ORB) long pattern</t>
         </is>
       </c>
-      <c r="N11" s="3" t="inlineStr">
+      <c r="P11" s="3" t="inlineStr">
         <is>
           <t>ASSUMED</t>
         </is>
       </c>
-      <c r="O11" s="3" t="inlineStr">
-        <is>
-          <t>Air-Way s135 only (double-pass 18 rows); M matches verified 6801 family; JIC/ORB ends inherit library verification</t>
-        </is>
-      </c>
-      <c r="P11" s="3" t="inlineStr"/>
-      <c r="Q11" t="inlineStr">
+      <c r="Q11" s="3" t="inlineStr">
+        <is>
+          <t>Air-Way s135 only (double-pass 18 rows); M matches verified 6801 family; JIC/ORB ends inherit library verification | ORB_I3 0.86 = Air-Way 6801 rows of the -08 ORB size (A5; I3 = Brennan 6801 / 6801-L / 6801-LL STEPs at -08) | ORB_THDL 0.344 = Air-Way 6801 rows of the -08 ORB size (A5; I3 = Brennan 6801 / 6801-L / 6801-LL STEPs at -08)</t>
+        </is>
+      </c>
+      <c r="R11" s="3" t="inlineStr">
+        <is>
+          <t>Brennan CAD record ORB leg M7 1.97 vs Air-Way M11 1.81 - built to Air-Way (Air-Way first; tell the user / OMi)</t>
+        </is>
+      </c>
+      <c r="S11" t="inlineStr">
         <is>
           <t>BUILD</t>
         </is>
       </c>
-      <c r="R11" t="inlineStr">
+      <c r="T11" t="inlineStr">
         <is>
           <t>6801-L-08-08-NWO-FG</t>
         </is>
@@ -1201,32 +1237,32 @@
       <c r="K12" s="3" t="n">
         <v>0.094</v>
       </c>
-      <c r="L12" s="3" t="inlineStr">
+      <c r="N12" s="3" t="inlineStr">
         <is>
           <t>6801-L-08-08-NWO</t>
         </is>
       </c>
-      <c r="M12" s="3" t="inlineStr">
+      <c r="O12" s="3" t="inlineStr">
         <is>
           <t>3/4-16 (JIC) x 3/4-16 (male ORB) long pattern</t>
         </is>
       </c>
-      <c r="N12" s="3" t="inlineStr">
+      <c r="P12" s="3" t="inlineStr">
         <is>
           <t>ASSUMED</t>
         </is>
       </c>
-      <c r="O12" s="3" t="inlineStr">
+      <c r="Q12" s="3" t="inlineStr">
         <is>
           <t>Air-Way s135 only (double-pass 18 rows); M matches verified 6801 family; JIC/ORB ends inherit library verification</t>
         </is>
       </c>
-      <c r="P12" s="3" t="inlineStr">
+      <c r="R12" s="3" t="inlineStr">
         <is>
           <t>DROP: no matching OMi SKU in catalog feed (2026-09-23)</t>
         </is>
       </c>
-      <c r="Q12" t="inlineStr">
+      <c r="S12" t="inlineStr">
         <is>
           <t>DROP</t>
         </is>
@@ -1268,32 +1304,32 @@
       <c r="K13" s="3" t="n">
         <v>0.107</v>
       </c>
-      <c r="L13" s="3" t="inlineStr">
+      <c r="N13" s="3" t="inlineStr">
         <is>
           <t>6801-L-08-10-NWO</t>
         </is>
       </c>
-      <c r="M13" s="3" t="inlineStr">
+      <c r="O13" s="3" t="inlineStr">
         <is>
           <t>3/4-16 (JIC) x 7/8-14 (male ORB) long pattern</t>
         </is>
       </c>
-      <c r="N13" s="3" t="inlineStr">
+      <c r="P13" s="3" t="inlineStr">
         <is>
           <t>ASSUMED</t>
         </is>
       </c>
-      <c r="O13" s="3" t="inlineStr">
+      <c r="Q13" s="3" t="inlineStr">
         <is>
           <t>Air-Way s135 only (double-pass 18 rows); M matches verified 6801 family; JIC/ORB ends inherit library verification</t>
         </is>
       </c>
-      <c r="P13" s="3" t="inlineStr">
+      <c r="R13" s="3" t="inlineStr">
         <is>
           <t>DROP: no matching OMi SKU in catalog feed (2026-09-23)</t>
         </is>
       </c>
-      <c r="Q13" t="inlineStr">
+      <c r="S13" t="inlineStr">
         <is>
           <t>DROP</t>
         </is>
@@ -1335,32 +1371,32 @@
       <c r="K14" s="3" t="n">
         <v>0.107</v>
       </c>
-      <c r="L14" s="3" t="inlineStr">
+      <c r="N14" s="3" t="inlineStr">
         <is>
           <t>6801-L-10-10-NWO-FG</t>
         </is>
       </c>
-      <c r="M14" s="3" t="inlineStr">
+      <c r="O14" s="3" t="inlineStr">
         <is>
           <t>7/8-14 (JIC) x 7/8-14 (male ORB) long pattern</t>
         </is>
       </c>
-      <c r="N14" s="3" t="inlineStr">
+      <c r="P14" s="3" t="inlineStr">
         <is>
           <t>ASSUMED</t>
         </is>
       </c>
-      <c r="O14" s="3" t="inlineStr">
+      <c r="Q14" s="3" t="inlineStr">
         <is>
           <t>Air-Way s135 only (double-pass 18 rows); M matches verified 6801 family; JIC/ORB ends inherit library verification</t>
         </is>
       </c>
-      <c r="P14" s="3" t="inlineStr">
+      <c r="R14" s="3" t="inlineStr">
         <is>
           <t>DROP: no matching OMi SKU in catalog feed (2026-09-23)</t>
         </is>
       </c>
-      <c r="Q14" t="inlineStr">
+      <c r="S14" t="inlineStr">
         <is>
           <t>DROP</t>
         </is>
@@ -1402,32 +1438,32 @@
       <c r="K15" s="3" t="n">
         <v>0.107</v>
       </c>
-      <c r="L15" s="3" t="inlineStr">
+      <c r="N15" s="3" t="inlineStr">
         <is>
           <t>6801-L-10-10-NWO</t>
         </is>
       </c>
-      <c r="M15" s="3" t="inlineStr">
+      <c r="O15" s="3" t="inlineStr">
         <is>
           <t>7/8-14 (JIC) x 7/8-14 (male ORB) long pattern</t>
         </is>
       </c>
-      <c r="N15" s="3" t="inlineStr">
+      <c r="P15" s="3" t="inlineStr">
         <is>
           <t>ASSUMED</t>
         </is>
       </c>
-      <c r="O15" s="3" t="inlineStr">
+      <c r="Q15" s="3" t="inlineStr">
         <is>
           <t>Air-Way s135 only (double-pass 18 rows); M matches verified 6801 family; JIC/ORB ends inherit library verification</t>
         </is>
       </c>
-      <c r="P15" s="3" t="inlineStr">
+      <c r="R15" s="3" t="inlineStr">
         <is>
           <t>DROP: no matching OMi SKU in catalog feed (2026-09-23)</t>
         </is>
       </c>
-      <c r="Q15" t="inlineStr">
+      <c r="S15" t="inlineStr">
         <is>
           <t>DROP</t>
         </is>
@@ -1469,32 +1505,32 @@
       <c r="K16" s="3" t="n">
         <v>0.125</v>
       </c>
-      <c r="L16" s="3" t="inlineStr">
+      <c r="N16" s="3" t="inlineStr">
         <is>
           <t>6801-L-10-12-NWO</t>
         </is>
       </c>
-      <c r="M16" s="3" t="inlineStr">
+      <c r="O16" s="3" t="inlineStr">
         <is>
           <t>7/8-14 (JIC) x 1 1/16-12 (male ORB) long pattern</t>
         </is>
       </c>
-      <c r="N16" s="3" t="inlineStr">
+      <c r="P16" s="3" t="inlineStr">
         <is>
           <t>ASSUMED</t>
         </is>
       </c>
-      <c r="O16" s="3" t="inlineStr">
+      <c r="Q16" s="3" t="inlineStr">
         <is>
           <t>Air-Way s135 only (double-pass 18 rows); M matches verified 6801 family; JIC/ORB ends inherit library verification</t>
         </is>
       </c>
-      <c r="P16" s="3" t="inlineStr">
+      <c r="R16" s="3" t="inlineStr">
         <is>
           <t>DROP: no matching OMi SKU in catalog feed (2026-09-23)</t>
         </is>
       </c>
-      <c r="Q16" t="inlineStr">
+      <c r="S16" t="inlineStr">
         <is>
           <t>DROP</t>
         </is>
@@ -1536,33 +1572,43 @@
       <c r="K17" s="3" t="n">
         <v>0.125</v>
       </c>
-      <c r="L17" s="3" t="inlineStr">
+      <c r="L17" t="n">
+        <v>1.14</v>
+      </c>
+      <c r="M17" t="n">
+        <v>0.469</v>
+      </c>
+      <c r="N17" s="3" t="inlineStr">
         <is>
           <t>6801-L-12-12-NWO-FG</t>
         </is>
       </c>
-      <c r="M17" s="3" t="inlineStr">
+      <c r="O17" s="3" t="inlineStr">
         <is>
           <t>1 1/16-12 (JIC) x 1 1/16-12 (male ORB) long pattern</t>
         </is>
       </c>
-      <c r="N17" s="3" t="inlineStr">
+      <c r="P17" s="3" t="inlineStr">
         <is>
           <t>ASSUMED</t>
         </is>
       </c>
-      <c r="O17" s="3" t="inlineStr">
-        <is>
-          <t>Air-Way s135 only (double-pass 18 rows); M matches verified 6801 family; JIC/ORB ends inherit library verification</t>
-        </is>
-      </c>
-      <c r="P17" s="3" t="inlineStr"/>
-      <c r="Q17" t="inlineStr">
+      <c r="Q17" s="3" t="inlineStr">
+        <is>
+          <t>Air-Way s135 only (double-pass 18 rows); M matches verified 6801 family; JIC/ORB ends inherit library verification | ORB_I3 1.14 = Air-Way 6801 rows of the -12 ORB size (A5; I3 = Brennan 6801 / 6801-L / 6801-LL STEPs at -08) | ORB_THDL 0.469 = Air-Way 6801 rows of the -12 ORB size (A5; I3 = Brennan 6801 / 6801-L / 6801-LL STEPs at -08)</t>
+        </is>
+      </c>
+      <c r="R17" s="3" t="inlineStr">
+        <is>
+          <t>Brennan CAD record ORB leg M7 2.62 vs Air-Way M11 2.47 - built to Air-Way (Air-Way first; tell the user / OMi)</t>
+        </is>
+      </c>
+      <c r="S17" t="inlineStr">
         <is>
           <t>BUILD</t>
         </is>
       </c>
-      <c r="R17" t="inlineStr">
+      <c r="T17" t="inlineStr">
         <is>
           <t>6801-L-12-12-NWO-FG</t>
         </is>
@@ -1604,32 +1650,32 @@
       <c r="K18" s="3" t="n">
         <v>0.125</v>
       </c>
-      <c r="L18" s="3" t="inlineStr">
+      <c r="N18" s="3" t="inlineStr">
         <is>
           <t>6801-L-12-12-NWO</t>
         </is>
       </c>
-      <c r="M18" s="3" t="inlineStr">
+      <c r="O18" s="3" t="inlineStr">
         <is>
           <t>1 1/16-12 (JIC) x 1 1/16-12 (male ORB) long pattern</t>
         </is>
       </c>
-      <c r="N18" s="3" t="inlineStr">
+      <c r="P18" s="3" t="inlineStr">
         <is>
           <t>ASSUMED</t>
         </is>
       </c>
-      <c r="O18" s="3" t="inlineStr">
+      <c r="Q18" s="3" t="inlineStr">
         <is>
           <t>Air-Way s135 only (double-pass 18 rows); M matches verified 6801 family; JIC/ORB ends inherit library verification</t>
         </is>
       </c>
-      <c r="P18" s="3" t="inlineStr">
+      <c r="R18" s="3" t="inlineStr">
         <is>
           <t>DROP: no matching OMi SKU in catalog feed (2026-09-23)</t>
         </is>
       </c>
-      <c r="Q18" t="inlineStr">
+      <c r="S18" t="inlineStr">
         <is>
           <t>DROP</t>
         </is>
@@ -1671,32 +1717,32 @@
       <c r="K19" s="3" t="n">
         <v>0.125</v>
       </c>
-      <c r="L19" s="3" t="inlineStr">
+      <c r="N19" s="3" t="inlineStr">
         <is>
           <t>6801-L-16-16-NWO</t>
         </is>
       </c>
-      <c r="M19" s="3" t="inlineStr">
+      <c r="O19" s="3" t="inlineStr">
         <is>
           <t>1 5/16-12 (JIC) x 1 5/16-12 (male ORB) long pattern</t>
         </is>
       </c>
-      <c r="N19" s="3" t="inlineStr">
+      <c r="P19" s="3" t="inlineStr">
         <is>
           <t>ASSUMED</t>
         </is>
       </c>
-      <c r="O19" s="3" t="inlineStr">
+      <c r="Q19" s="3" t="inlineStr">
         <is>
           <t>Air-Way s135 only (double-pass 18 rows); M matches verified 6801 family; JIC/ORB ends inherit library verification</t>
         </is>
       </c>
-      <c r="P19" s="3" t="inlineStr">
+      <c r="R19" s="3" t="inlineStr">
         <is>
           <t>DROP: no matching OMi SKU in catalog feed (2026-09-23) | near-match donor for OMi SKU 6801-L-16-16-NWO-FG</t>
         </is>
       </c>
-      <c r="Q19" t="inlineStr">
+      <c r="S19" t="inlineStr">
         <is>
           <t>DROP</t>
         </is>
@@ -1738,32 +1784,32 @@
       <c r="K20" s="3" t="n">
         <v>0.125</v>
       </c>
-      <c r="L20" s="3" t="inlineStr">
+      <c r="N20" s="3" t="inlineStr">
         <is>
           <t>6801-L-20-20-NWO</t>
         </is>
       </c>
-      <c r="M20" s="3" t="inlineStr">
+      <c r="O20" s="3" t="inlineStr">
         <is>
           <t>1 5/8-12 (JIC) x 1 5/8-12 (male ORB) long pattern</t>
         </is>
       </c>
-      <c r="N20" s="3" t="inlineStr">
+      <c r="P20" s="3" t="inlineStr">
         <is>
           <t>ASSUMED</t>
         </is>
       </c>
-      <c r="O20" s="3" t="inlineStr">
+      <c r="Q20" s="3" t="inlineStr">
         <is>
           <t>Air-Way s135 only (double-pass 18 rows); M matches verified 6801 family; JIC/ORB ends inherit library verification</t>
         </is>
       </c>
-      <c r="P20" s="3" t="inlineStr">
+      <c r="R20" s="3" t="inlineStr">
         <is>
           <t>DROP: no matching OMi SKU in catalog feed (2026-09-23) | near-match donor for OMi SKU 6801-L-20-20-NWO-FG</t>
         </is>
       </c>
-      <c r="Q20" t="inlineStr">
+      <c r="S20" t="inlineStr">
         <is>
           <t>DROP</t>
         </is>
@@ -1778,46 +1824,67 @@
       <c r="B21" t="n">
         <v>1.81</v>
       </c>
+      <c r="C21" t="n">
+        <v>3.06</v>
+      </c>
       <c r="D21" t="n">
         <v>1.5</v>
       </c>
       <c r="E21" t="n">
         <v>1.312</v>
       </c>
+      <c r="F21" t="n">
+        <v>0.844</v>
+      </c>
+      <c r="G21" t="n">
+        <v>0.844</v>
+      </c>
+      <c r="H21" t="n">
+        <v>1.3125</v>
+      </c>
+      <c r="I21" t="n">
+        <v>1.3125</v>
+      </c>
       <c r="J21" t="n">
         <v>1.195</v>
       </c>
-      <c r="L21" t="inlineStr">
+      <c r="L21" t="n">
+        <v>1.14</v>
+      </c>
+      <c r="M21" t="n">
+        <v>0.469</v>
+      </c>
+      <c r="N21" t="inlineStr">
         <is>
           <t>6801-L-16-16-NWO-FG</t>
         </is>
       </c>
-      <c r="N21" t="inlineStr">
+      <c r="P21" t="inlineStr">
         <is>
           <t>ASSUMED</t>
         </is>
       </c>
-      <c r="O21" t="inlineStr">
-        <is>
-          <t>[BRENNAN-CAD 2026-10-21: C4HEX@HEX, M@DRIVE, ORB_GRVDIA@DRIVE, Y@REF] OMi catalog SKU (omindustrial.com collections feed (cs-adapters, carbon-steel-flange-adapters-accessories, carbon-steel-braze-beaded-hose; products.json limit=50, single pass 2026-09-23)); Air-Way has this size only as 6801-L-16-16-NWO (differs by -FG/-UNPL suffix) -&gt; dims NOT copied</t>
-        </is>
-      </c>
-      <c r="P21" t="inlineStr">
-        <is>
-          <t>BUILD-NEAR: forged (-FG) and non-FG variants differ in length on other series, so 6801-L-16-16-NWO dims are NOT assumed; confirm before modelling | Brennan CAD record 6801-L-16-16-NWO-FG (PARTcommunity / CADENAS, C4HEX@HEX=C, M@DRIVE=M, ORB_GRVDIA@DRIVE=HT, Y@REF=Y; user 2026-10-21 "yes you can use them following my rule")</t>
-        </is>
-      </c>
       <c r="Q21" t="inlineStr">
         <is>
+          <t>[BRENNAN-CAD 2026-10-21 group B: M11@DRIVE, D1@BORE, D2@BORE] [BRENNAN-CAD 2026-10-21: C4HEX@HEX, M@DRIVE, ORB_GRVDIA@DRIVE, Y@REF] OMi catalog SKU (omindustrial.com collections feed (cs-adapters, carbon-steel-flange-adapters-accessories, carbon-steel-braze-beaded-hose; products.json limit=50, single pass 2026-09-23)); Air-Way has this size only as 6801-L-16-16-NWO (differs by -FG/-UNPL suffix) -&gt; dims NOT copied | ORB_I3 1.14 = Air-Way 6801 rows of the -16 ORB size (A5; I3 = Brennan 6801 / 6801-L / 6801-LL STEPs at -08) | ORB_THDL 0.469 = Air-Way 6801 rows of the -16 ORB size (A5; I3 = Brennan 6801 / 6801-L / 6801-LL STEPs at -08)</t>
+        </is>
+      </c>
+      <c r="R21" t="inlineStr">
+        <is>
+          <t>BUILD-NEAR: forged (-FG) and non-FG variants differ in length on other series, so 6801-L-16-16-NWO dims are NOT assumed; confirm before modelling | Brennan CAD record 6801-L-16-16-NWO-FG (PARTcommunity / CADENAS, C4HEX@HEX=C, M@DRIVE=M, ORB_GRVDIA@DRIVE=HT, Y@REF=Y; user 2026-10-21 "yes you can use them following my rule") | Brennan CAD record 6801-L-16-16-NWO-FG (PARTcommunity / CADENAS, group B 2026-10-21: M11@DRIVE=M7, D1@BORE=B1D, D2@BORE=B2D; user 2026-10-21 "yes you can use them following my rule")</t>
+        </is>
+      </c>
+      <c r="S21" t="inlineStr">
+        <is>
           <t>BUILD</t>
         </is>
       </c>
-      <c r="R21" t="inlineStr">
+      <c r="T21" t="inlineStr">
         <is>
           <t>6801-L-16-16-NWO-FG</t>
         </is>
       </c>
-      <c r="S21" t="inlineStr">
+      <c r="U21" t="inlineStr">
         <is>
           <t>BRENNAN</t>
         </is>
@@ -1832,46 +1899,67 @@
       <c r="B22" t="n">
         <v>2.06</v>
       </c>
+      <c r="C22" t="n">
+        <v>3.48</v>
+      </c>
       <c r="D22" t="n">
         <v>1.875</v>
       </c>
       <c r="E22" t="n">
         <v>1.625</v>
       </c>
+      <c r="F22" t="n">
+        <v>1.078</v>
+      </c>
+      <c r="G22" t="n">
+        <v>1.078</v>
+      </c>
+      <c r="H22" t="n">
+        <v>1.625</v>
+      </c>
+      <c r="I22" t="n">
+        <v>1.625</v>
+      </c>
       <c r="J22" t="n">
         <v>1.507</v>
       </c>
-      <c r="L22" t="inlineStr">
+      <c r="L22" t="n">
+        <v>1.14</v>
+      </c>
+      <c r="M22" t="n">
+        <v>0.469</v>
+      </c>
+      <c r="N22" t="inlineStr">
         <is>
           <t>6801-L-20-20-NWO-FG</t>
         </is>
       </c>
-      <c r="N22" t="inlineStr">
+      <c r="P22" t="inlineStr">
         <is>
           <t>ASSUMED</t>
         </is>
       </c>
-      <c r="O22" t="inlineStr">
-        <is>
-          <t>[BRENNAN-CAD 2026-10-21: C4HEX@HEX, M@DRIVE, ORB_GRVDIA@DRIVE, Y@REF] OMi catalog SKU (omindustrial.com collections feed (cs-adapters, carbon-steel-flange-adapters-accessories, carbon-steel-braze-beaded-hose; products.json limit=50, single pass 2026-09-23)); Air-Way has this size only as 6801-L-20-20-NWO (differs by -FG/-UNPL suffix) -&gt; dims NOT copied</t>
-        </is>
-      </c>
-      <c r="P22" t="inlineStr">
-        <is>
-          <t>BUILD-NEAR: forged (-FG) and non-FG variants differ in length on other series, so 6801-L-20-20-NWO dims are NOT assumed; confirm before modelling | Brennan CAD record 6801-L-20-20-NWO-FG (PARTcommunity / CADENAS, C4HEX@HEX=C, M@DRIVE=M, ORB_GRVDIA@DRIVE=HT, Y@REF=Y; user 2026-10-21 "yes you can use them following my rule")</t>
-        </is>
-      </c>
       <c r="Q22" t="inlineStr">
         <is>
+          <t>[BRENNAN-CAD 2026-10-21 group B: M11@DRIVE, D1@BORE, D2@BORE] [BRENNAN-CAD 2026-10-21: C4HEX@HEX, M@DRIVE, ORB_GRVDIA@DRIVE, Y@REF] OMi catalog SKU (omindustrial.com collections feed (cs-adapters, carbon-steel-flange-adapters-accessories, carbon-steel-braze-beaded-hose; products.json limit=50, single pass 2026-09-23)); Air-Way has this size only as 6801-L-20-20-NWO (differs by -FG/-UNPL suffix) -&gt; dims NOT copied | ORB_I3 1.14 = Air-Way 6801 rows of the -20 ORB size (A5; I3 = Brennan 6801 / 6801-L / 6801-LL STEPs at -08) | ORB_THDL 0.469 = Air-Way 6801 rows of the -20 ORB size (A5; I3 = Brennan 6801 / 6801-L / 6801-LL STEPs at -08)</t>
+        </is>
+      </c>
+      <c r="R22" t="inlineStr">
+        <is>
+          <t>BUILD-NEAR: forged (-FG) and non-FG variants differ in length on other series, so 6801-L-20-20-NWO dims are NOT assumed; confirm before modelling | Brennan CAD record 6801-L-20-20-NWO-FG (PARTcommunity / CADENAS, C4HEX@HEX=C, M@DRIVE=M, ORB_GRVDIA@DRIVE=HT, Y@REF=Y; user 2026-10-21 "yes you can use them following my rule") | Brennan CAD record 6801-L-20-20-NWO-FG (PARTcommunity / CADENAS, group B 2026-10-21: M11@DRIVE=M7, D1@BORE=B1D, D2@BORE=B2D; user 2026-10-21 "yes you can use them following my rule")</t>
+        </is>
+      </c>
+      <c r="S22" t="inlineStr">
+        <is>
           <t>BUILD</t>
         </is>
       </c>
-      <c r="R22" t="inlineStr">
+      <c r="T22" t="inlineStr">
         <is>
           <t>6801-L-20-20-NWO-FG</t>
         </is>
       </c>
-      <c r="S22" t="inlineStr">
+      <c r="U22" t="inlineStr">
         <is>
           <t>BRENNAN</t>
         </is>

</xml_diff>